<commit_message>
changes to write to all sheets
</commit_message>
<xml_diff>
--- a/files/processed_data/pokemon_cards_processed.xlsx
+++ b/files/processed_data/pokemon_cards_processed.xlsx
@@ -7,7 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="purchase" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="card" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="card_instance" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="card_grade" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="seller" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="purchase" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,6 +421,2070 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>card_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>row_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>card_set_id</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>card_holo_flag</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>card_first_edition_flag</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>card_promo_flag</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>card_language_id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>card_rarity_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>extra_details</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>card_image_reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Dark Blastoise</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>{'detail_1': 'Lightly Played', 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Togetic</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>11</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>{'detail_1': None, 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Charizard</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>{'detail_1': None, 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Charizard</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>{'detail_1': None, 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Charmander</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>{'detail_1': '4th Print', 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Squirtle</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>16</v>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>{'detail_1': None, 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Typhlosion</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>11</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>{'detail_1': None, 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Pikachu</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="b">
+        <v>0</v>
+      </c>
+      <c r="F9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G9" t="b">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>{'detail_1': 'Yellow Cheeks', 'detail_2': '4th Print', 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Pikachu</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" t="b">
+        <v>0</v>
+      </c>
+      <c r="G10" t="b">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>{'detail_1': 'Yellow Cheeks', 'detail_2': 'Shadowless', 'detail_3': '4th Print'}</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Houndoom</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>10</v>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>{'detail_1': None, 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Dark Alakazam</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>14</v>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" t="b">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>{'detail_1': None, 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Radiant Blastoise</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>12</v>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G13" t="b">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>{'detail_1': None, 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Raichu</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G14" t="b">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>{'detail_1': None, 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Squirtle</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G15" t="b">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>{'detail_1': '4th Print', 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Arcanine</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+      <c r="F16" t="b">
+        <v>1</v>
+      </c>
+      <c r="G16" t="b">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>{'detail_1': None, 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Blastoise</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>7</v>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" t="b">
+        <v>1</v>
+      </c>
+      <c r="G17" t="b">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>{'detail_1': None, 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Dark Weezing</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>14</v>
+      </c>
+      <c r="E18" t="b">
+        <v>1</v>
+      </c>
+      <c r="F18" t="b">
+        <v>1</v>
+      </c>
+      <c r="G18" t="b">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>{'detail_1': None, 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Magneton</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E19" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" t="b">
+        <v>0</v>
+      </c>
+      <c r="G19" t="b">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>{'detail_1': None, 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Charizard</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>8</v>
+      </c>
+      <c r="E20" t="b">
+        <v>0</v>
+      </c>
+      <c r="F20" t="b">
+        <v>0</v>
+      </c>
+      <c r="G20" t="b">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>2</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>{'detail_1': 'Grand Prix Illustrator', 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Radiant Charizard</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>9</v>
+      </c>
+      <c r="E21" t="b">
+        <v>1</v>
+      </c>
+      <c r="F21" t="b">
+        <v>0</v>
+      </c>
+      <c r="G21" t="b">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>2</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>{'detail_1': 'VSTAR Universe', 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Radiant Venasaur</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>13</v>
+      </c>
+      <c r="E22" t="b">
+        <v>1</v>
+      </c>
+      <c r="F22" t="b">
+        <v>0</v>
+      </c>
+      <c r="G22" t="b">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>{'detail_1': None, 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Golem</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" t="b">
+        <v>0</v>
+      </c>
+      <c r="F23" t="b">
+        <v>1</v>
+      </c>
+      <c r="G23" t="b">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" t="n">
+        <v>2</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>{'detail_1': None, 'detail_2': None, 'detail_3': None}</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>card_instance_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>row_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>card_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" t="n">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>grade_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>card_instance_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>row_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>grade_description_id</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>grading_certification_number</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>graded_card_url</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>123.0</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>456.0</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>789.0</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1122.0</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1455.0</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1788.0</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>8</v>
+      </c>
+      <c r="C8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2121.0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>9</v>
+      </c>
+      <c r="C9" t="n">
+        <v>9</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2454.0</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>10</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2787.0</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>11</v>
+      </c>
+      <c r="C11" t="n">
+        <v>11</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>3120.0</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>12</v>
+      </c>
+      <c r="C12" t="n">
+        <v>12</v>
+      </c>
+      <c r="D12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>3453.0</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>13</v>
+      </c>
+      <c r="C13" t="n">
+        <v>13</v>
+      </c>
+      <c r="D13" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>3786.0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>14</v>
+      </c>
+      <c r="C14" t="n">
+        <v>14</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>4119.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>15</v>
+      </c>
+      <c r="C15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D15" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>4452.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>16</v>
+      </c>
+      <c r="C16" t="n">
+        <v>16</v>
+      </c>
+      <c r="D16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>4785.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>17</v>
+      </c>
+      <c r="C17" t="n">
+        <v>17</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>5118.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>18</v>
+      </c>
+      <c r="C18" t="n">
+        <v>18</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>5451.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>19</v>
+      </c>
+      <c r="C19" t="n">
+        <v>19</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>5784.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>20</v>
+      </c>
+      <c r="C20" t="n">
+        <v>20</v>
+      </c>
+      <c r="D20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>6117.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>21</v>
+      </c>
+      <c r="C21" t="n">
+        <v>21</v>
+      </c>
+      <c r="D21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>6450.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>22</v>
+      </c>
+      <c r="C22" t="n">
+        <v>22</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>6783.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>seller_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>row_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>seller</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>country_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>The Brotherhood Games</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://thebrotherhoodgames.co.uk/products/Pokemon-c160349505</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>coco_mew</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>emanator88</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>smithydaniel19</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>wilson406</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>andearn-36</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>cardmastersuk</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>rorye94</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>gokujjr</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>calsharcollectables</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>rob145558</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>wickfordcards</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>purpleoblivion</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>j_a_cards</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ascendancecollectibles</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>wookiewhiskers</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>tcec0308</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>d-tcg112</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>poke_phd</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>drphilcards3</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>cardstoreuk</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://ebay.co.uk</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
dim table reads added for excel output
</commit_message>
<xml_diff>
--- a/files/processed_data/pokemon_cards_processed.xlsx
+++ b/files/processed_data/pokemon_cards_processed.xlsx
@@ -12,6 +12,14 @@
     <sheet name="card_grade" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="seller" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="purchase" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="card_set" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="language" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="rarity" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="grading_company" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="grade_description" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="currency" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="purchase_source" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="country" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,6 +431,19 @@
   </sheetPr>
   <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="82" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1294,6 +1315,264 @@
         </is>
       </c>
       <c r="K23" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>grade_description_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>grading_company_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>grade</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>grade_description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Gem Mint</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NM-Mint</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Gem Mint</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Gem Mint</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="n">
+        <v>9</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Mint</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>currency_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>currency_code</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>purchase_source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Comic-Con</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>eBay</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>country_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1308,6 +1587,11 @@
   </sheetPr>
   <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1581,6 +1865,14 @@
   </sheetPr>
   <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2047,6 +2339,13 @@
   </sheetPr>
   <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="63" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2487,6 +2786,19 @@
   </sheetPr>
   <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3274,6 +3586,483 @@
       </c>
       <c r="K22" s="1" t="n">
         <v>45533</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>card_set_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Base Set</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1999-2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bonds To The End Of Time</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Elite Trainer Box</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Flight of Legends</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1999</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Hollow Shining Darkness</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>JPN S-P</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>JPN SWSH</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Neo 2</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Neo Genesis</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Pokémon Go</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pokémon Go JPN</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Team Rocket</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>language_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rarity_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>rarity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Illustrator Rare</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>grading_company_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>company_full_name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PokeGrade</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ace</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ace Grading Company</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>